<commit_message>
BOQ multi-select, fixed rows, mandatory, and warranty sync
</commit_message>
<xml_diff>
--- a/BOQ Sequence.xlsx
+++ b/BOQ Sequence.xlsx
@@ -1,37 +1,45 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Welcome\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\My Drive\SAK-IT\014 - EPC Solar\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{752B7E64-7E9D-4A27-9F6C-99E98CD076E4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CA954026-FC93-460E-A234-44B509FA4261}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{9FEFEE0D-5BF3-42F3-9843-05ED026296D5}"/>
+    <workbookView xWindow="10185" yWindow="-15" windowWidth="10320" windowHeight="10950" xr2:uid="{9FEFEE0D-5BF3-42F3-9843-05ED026296D5}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet2" sheetId="2" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet2!$A$1:$B$21</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet2!$A$1:$B$22</definedName>
   </definedNames>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="22">
-  <si>
-    <t>Row Labels</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="36">
   <si>
     <t>AC CABLE</t>
   </si>
@@ -94,13 +102,58 @@
   </si>
   <si>
     <t>Sequence</t>
+  </si>
+  <si>
+    <t>Mandatory</t>
+  </si>
+  <si>
+    <t>Multiple</t>
+  </si>
+  <si>
+    <t>Yes</t>
+  </si>
+  <si>
+    <t>No</t>
+  </si>
+  <si>
+    <t>AC DISTRIBUTION BOX</t>
+  </si>
+  <si>
+    <t>DC DISTRIBUTION BOX</t>
+  </si>
+  <si>
+    <t>Fixed</t>
+  </si>
+  <si>
+    <t>ITEM TYPE</t>
+  </si>
+  <si>
+    <t>ITEM HEAD</t>
+  </si>
+  <si>
+    <t>YEs</t>
+  </si>
+  <si>
+    <t>yes</t>
+  </si>
+  <si>
+    <t>no</t>
+  </si>
+  <si>
+    <t>TRANSPORTATION</t>
+  </si>
+  <si>
+    <t>INSTALLATION &amp; COMMISSIONING</t>
+  </si>
+  <si>
+    <t>fixed</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -108,16 +161,43 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri Light"/>
+      <family val="2"/>
+      <scheme val="major"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0" tint="-0.14999847407452621"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -125,12 +205,46 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -411,184 +525,376 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CD3DFB50-4A6A-4E74-8108-6D4E1DB14305}">
-  <dimension ref="A1:B21"/>
+  <dimension ref="A1:E24"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
+    <col min="1" max="1" width="9.140625" style="1"/>
     <col min="2" max="2" width="38.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="17.85546875" customWidth="1"/>
+    <col min="4" max="4" width="10.7109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="9.140625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="D1" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="B1" t="s">
+      <c r="E1" s="2" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2" s="3">
+        <v>1</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="C2" s="4"/>
+      <c r="D2" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A3" s="3">
+        <v>2</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="C3" s="4"/>
+      <c r="D3" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4" s="3">
+        <v>3</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="C4" s="4"/>
+      <c r="D4" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A5" s="3">
+        <v>4</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="C5" s="4"/>
+      <c r="D5" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="E5" s="3" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A6" s="3">
+        <v>5</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="D6" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="E6" s="3" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A7" s="3"/>
+      <c r="B7" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="D7" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="E7" s="3" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A8" s="3">
+        <v>6</v>
+      </c>
+      <c r="B8" s="4" t="s">
         <v>0</v>
       </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A2">
+      <c r="C8" s="4"/>
+      <c r="D8" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="E8" s="3" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A9" s="3">
+        <v>7</v>
+      </c>
+      <c r="B9" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="C9" s="4"/>
+      <c r="D9" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="E9" s="3" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A10" s="3">
+        <v>8</v>
+      </c>
+      <c r="B10" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="C10" s="4"/>
+      <c r="D10" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="E10" s="3" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A11" s="3">
+        <v>9</v>
+      </c>
+      <c r="B11" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="C11" s="4"/>
+      <c r="D11" s="5" t="s">
+        <v>32</v>
+      </c>
+      <c r="E11" s="3" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A12" s="3">
+        <v>10</v>
+      </c>
+      <c r="B12" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="C12" s="4"/>
+      <c r="D12" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="E12" s="3" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A13" s="3">
+        <v>11</v>
+      </c>
+      <c r="B13" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="C13" s="4"/>
+      <c r="D13" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="E13" s="3" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A14" s="3">
+        <v>12</v>
+      </c>
+      <c r="B14" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C14" s="4"/>
+      <c r="D14" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="E14" s="3" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A15" s="3">
+        <v>13</v>
+      </c>
+      <c r="B15" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="C15" s="4"/>
+      <c r="D15" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="E15" s="3" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A16" s="3">
+        <v>14</v>
+      </c>
+      <c r="B16" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C16" s="4"/>
+      <c r="D16" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="E16" s="3" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A17" s="3">
+        <v>15</v>
+      </c>
+      <c r="B17" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="C17" s="4"/>
+      <c r="D17" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="E17" s="3" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A18" s="3">
+        <v>16</v>
+      </c>
+      <c r="B18" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="C18" s="4"/>
+      <c r="D18" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="E18" s="3" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A19" s="3">
+        <v>17</v>
+      </c>
+      <c r="B19" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="C19" s="4"/>
+      <c r="D19" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="E19" s="3" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A20" s="3">
+        <v>18</v>
+      </c>
+      <c r="B20" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="C20" s="6"/>
+      <c r="D20" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="E20" s="3" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A21" s="3">
+        <v>19</v>
+      </c>
+      <c r="B21" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="C21" s="4"/>
+      <c r="D21" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="E21" s="3" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A22" s="3">
+        <v>20</v>
+      </c>
+      <c r="B22" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="B2" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A3">
-        <v>2</v>
-      </c>
-      <c r="B3" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A4">
-        <v>3</v>
-      </c>
-      <c r="B4" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A5">
-        <v>4</v>
-      </c>
-      <c r="B5" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A6">
-        <v>5</v>
-      </c>
-      <c r="B6" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A7">
-        <v>6</v>
-      </c>
-      <c r="B7" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A8">
-        <v>7</v>
-      </c>
-      <c r="B8" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A9">
-        <v>8</v>
-      </c>
-      <c r="B9" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A10">
-        <v>9</v>
-      </c>
-      <c r="B10" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A11">
-        <v>10</v>
-      </c>
-      <c r="B11" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A12">
-        <v>11</v>
-      </c>
-      <c r="B12" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A13">
-        <v>12</v>
-      </c>
-      <c r="B13" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A14">
-        <v>13</v>
-      </c>
-      <c r="B14" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A15">
-        <v>14</v>
-      </c>
-      <c r="B15" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A16">
-        <v>15</v>
-      </c>
-      <c r="B16" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A17">
-        <v>16</v>
-      </c>
-      <c r="B17" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A18">
-        <v>17</v>
-      </c>
-      <c r="B18" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A19">
-        <v>18</v>
-      </c>
-      <c r="B19" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A20">
-        <v>19</v>
-      </c>
-      <c r="B20" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A21">
-        <v>20</v>
-      </c>
-      <c r="B21" t="s">
-        <v>2</v>
+      <c r="C22" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="D22" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="E22" s="3" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A23" s="3"/>
+      <c r="B23" s="4"/>
+      <c r="C23" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="D23" s="3"/>
+      <c r="E23" s="3" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A24" s="3"/>
+      <c r="B24" s="4"/>
+      <c r="C24" s="4"/>
+      <c r="D24" s="3"/>
+      <c r="E24" s="3" t="s">
+        <v>31</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:B21" xr:uid="{CD3DFB50-4A6A-4E74-8108-6D4E1DB14305}">
-    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:B21">
-      <sortCondition ref="A1:A21"/>
+  <autoFilter ref="A1:B22" xr:uid="{CD3DFB50-4A6A-4E74-8108-6D4E1DB14305}">
+    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:B22">
+      <sortCondition ref="A1:A22"/>
     </sortState>
   </autoFilter>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>